<commit_message>
refactor(ui): update dashboard account and admin plans to light theme, fix auth redirect and tool routings
</commit_message>
<xml_diff>
--- a/pricing.xlsx
+++ b/pricing.xlsx
@@ -1,26 +1,155 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackn\spyder\dangtinbds\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F03621F4-AB34-41E1-AB56-C851E0150069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+  <si>
+    <t>Biến số</t>
+  </si>
+  <si>
+    <t>Mức 1 (Thấp)</t>
+  </si>
+  <si>
+    <t>Mức 2 (Trung bình)</t>
+  </si>
+  <si>
+    <t>Mức 3 (Cao)</t>
+  </si>
+  <si>
+    <t>Credit ($C$)</t>
+  </si>
+  <si>
+    <t>Hệ số $\delta_c$</t>
+  </si>
+  <si>
+    <t>Thời gian ($T$)</t>
+  </si>
+  <si>
+    <t>30 ngày</t>
+  </si>
+  <si>
+    <t>60 ngày</t>
+  </si>
+  <si>
+    <t>90 ngày</t>
+  </si>
+  <si>
+    <t>Hệ số $\delta_t$</t>
+  </si>
+  <si>
+    <t>1.0 (Không giảm)</t>
+  </si>
+  <si>
+    <t>0.9 (Giảm 10%)</t>
+  </si>
+  <si>
+    <t>0.8 (Giảm 20%)</t>
+  </si>
+  <si>
+    <t>0.85 (Giảm 15%)</t>
+  </si>
+  <si>
+    <t>0.75 (Giảm 25%)</t>
+  </si>
+  <si>
+    <t>Credits \ Thời gian</t>
+  </si>
+  <si>
+    <t>30 Ngày</t>
+  </si>
+  <si>
+    <t>60 Ngày</t>
+  </si>
+  <si>
+    <t>90 Ngày</t>
+  </si>
+  <si>
+    <t>1.000 Credits</t>
+  </si>
+  <si>
+    <t>155.000đ</t>
+  </si>
+  <si>
+    <t>219.000đ</t>
+  </si>
+  <si>
+    <t>255.000đ</t>
+  </si>
+  <si>
+    <t>3.500 Credits</t>
+  </si>
+  <si>
+    <t>299.000đ</t>
+  </si>
+  <si>
+    <t>359.000đ</t>
+  </si>
+  <si>
+    <t>399.000đ</t>
+  </si>
+  <si>
+    <t>10.000 Credits</t>
+  </si>
+  <si>
+    <t>649.000đ</t>
+  </si>
+  <si>
+    <t>719.000đ</t>
+  </si>
+  <si>
+    <t>789.000đ</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="169" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -46,13 +175,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +462,228 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C1">
+        <v>1</v>
+      </c>
+      <c r="D1">
+        <v>0.9</v>
+      </c>
+      <c r="E1">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <v>1000</v>
+      </c>
+      <c r="D2">
+        <v>3500</v>
+      </c>
+      <c r="E2">
+        <v>10000</v>
+      </c>
+      <c r="F2">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>30</v>
+      </c>
+      <c r="C3" s="1">
+        <f>C$2*$F$2*C$1+$B3*$A3*$B$6</f>
+        <v>155000</v>
+      </c>
+      <c r="D3" s="1">
+        <f t="shared" ref="D3:E5" si="0">D$2*$F$2*D$1+$B3*$A3*$B$6</f>
+        <v>294750</v>
+      </c>
+      <c r="E3" s="1">
+        <f t="shared" si="0"/>
+        <v>610000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0.85</v>
+      </c>
+      <c r="B4">
+        <v>60</v>
+      </c>
+      <c r="C4" s="1">
+        <f t="shared" ref="C4:C5" si="1">C$2*$F$2*C$1+$B4*$A4*$B$6</f>
+        <v>218000</v>
+      </c>
+      <c r="D4" s="1">
+        <f t="shared" si="0"/>
+        <v>357750</v>
+      </c>
+      <c r="E4" s="1">
+        <f t="shared" si="0"/>
+        <v>673000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>0.75</v>
+      </c>
+      <c r="B5">
+        <v>90</v>
+      </c>
+      <c r="C5" s="1">
+        <f t="shared" si="1"/>
+        <v>267500</v>
+      </c>
+      <c r="D5" s="1">
+        <f t="shared" si="0"/>
+        <v>407250</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" si="0"/>
+        <v>722500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B6">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>0</v>
+      </c>
+      <c r="I9" t="s">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>2</v>
+      </c>
+      <c r="K9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>4</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>3.5</v>
+      </c>
+      <c r="K10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="H11" t="s">
+        <v>5</v>
+      </c>
+      <c r="I11" t="s">
+        <v>11</v>
+      </c>
+      <c r="J11" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I12" t="s">
+        <v>7</v>
+      </c>
+      <c r="J12" t="s">
+        <v>8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I13" t="s">
+        <v>11</v>
+      </c>
+      <c r="J13" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>